<commit_message>
CI on 3.10 and 3.13, and one script to run the checks anywhere
`./check.sh` runs the unit tests and all 60 validators offline, and prints the
output only of the ones that failed. The same script runs in CI and on a laptop,
so the command that gates a push is the command you can run before making one.

The workflow installs the PACKAGE rather than the checkout -- `pip install .`,
then `quadrium --help`, then the checks, then the shipped example end to end --
because a package that imports from a checkout but does not install is a package
nobody can use. Both 3.10 and 3.13, since `requires-python = ">=3.10"` is a
promise. It also runs weekly, to catch numpy or openpyxl moving underneath.

Also: the shipped example's own instructions named a script retired at the
rename, and are regenerated.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/configs/ejemplo.xlsx
+++ b/configs/ejemplo.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -512,35 +512,126 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t># table_kind: uk_analytical (the ONS workbook) or interchange</t>
+          <t># table_kind: uk_analytical  the ONS workbook (industry x industry)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>#             (the project's own format, see io_loader).</t>
+          <t>#             ine_interior  the INE workbook, domestic output</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>#</t>
+          <t>#             ine_total     the INE workbook, total flows</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t># Fill in the other sheets, then run:</t>
+          <t>#             interchange   the project's own format, and what</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>#     python3 run_iofoundry.py &lt;this file&gt;</t>
+          <t>#                           this engine writes -- point at a</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>#                           result to split a second sector.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>#             eurostat      downloaded by country and year.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t># For table_kind: eurostat, delete table_path (or use it to say</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t># where to cache) and add instead:</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>#     eurostat_geo       ES        two-letter country code</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>#     eurostat_year      2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>#     eurostat_dataset   product_by_product | industry_by_industry</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>#     eurostat_variant   domestic | total</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t># Fill in the other sheets, then run:</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>#     quadrium &lt;this file&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t># (from a checkout, without installing: python3 run_quadrium.py)</t>
         </is>
       </c>
     </row>

</xml_diff>